<commit_message>
HF publication review: fix leaks, normalize names, package for upload
- Remove answer leakage: drop 10 definition questions whose term appears
  in the question (incl. via the statute title) and the 7 trivial
  law-type questions (identical answers); refill from article-locate
- Normalize product names shared between KB and benchmark: collapse
  newlines/whitespace from raw FSS names, and append credit type
  qualifiers only on real (bank, name) collisions — fixes double
  parentheses like "가계신용대출(일반)(일반신용대출)"
- Korean particle selection (을/를) by final consonant in article
  questions; unit field always present for stable pyarrow schema
- Verified: zero leaks/newlines/duplicates, datasets.load_dataset
  round-trip, all 24 tests pass, benchmark unchanged at 83/98/99
- dist/hf-bank-onto-bench/: upload-ready HF repo (README with configs
  YAML + data/test.jsonl), dataset card records the review history

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/bank-onto-benchmark-v1.xlsx
+++ b/docs/bank-onto-benchmark-v1.xlsx
@@ -2079,17 +2079,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>BNK더조은정기예금 || IBK굴리기통장(정기예금) || IBK더굴리기통장(실세금리정기예금) || IBK평생한가족통장(실세금리정기예금) || JB 123 정기예금
- (만기일시지급식) || JB 다이렉트예금통장
-(만기일시지급식) || J정기예금
-(만기지급식) || KB Star 정기예금 || KDB 정기예금 || LIVE정기예금 || NH고향사랑기부예금 || NH내가Green초록세상예금 || NH올원e예금 || NH왈츠회전예금 II || Sh첫만남우대예금 || Sh해양플라스틱Zero!예금
-(만기일시지급식) || The든든예금(시즌2) || The파트너예금 || The플러스예금 || WON플러스예금 || e-그린세이브예금 || iM스마트예금 || iM함께예금 || 굿스타트예금 || 내맘 쏙 정기예금 || 더(The) 레벨업 정기예금 || 더(The) 특판 정기예금 || 미즈월복리정기예금 || 스마일드림 
-정기예금
-(개인/선이자
-지급식) || 스마트모아Dream정기예금 || 신한My플러스 정기예금 || 쏠편한 정기예금 || 제주Dream
-정기예금
-(개인/만기
-지급식) || 카카오뱅크 정기예금 || 코드K 정기예금 || 토스뱅크 먼저 이자 받는 정기예금 || 하나의정기예금 || 헤이(Hey)정기예금</t>
+          <t>BNK더조은정기예금 || IBK굴리기통장(정기예금) || IBK더굴리기통장(실세금리정기예금) || IBK평생한가족통장(실세금리정기예금) || JB 123 정기예금 (만기일시지급식) || JB 다이렉트예금통장 (만기일시지급식) || J정기예금 (만기지급식) || KB Star 정기예금 || KDB 정기예금 || LIVE정기예금 || NH고향사랑기부예금 || NH내가Green초록세상예금 || NH올원e예금 || NH왈츠회전예금 II || Sh첫만남우대예금 || Sh해양플라스틱Zero!예금 (만기일시지급식) || The든든예금(시즌2) || The파트너예금 || The플러스예금 || WON플러스예금 || e-그린세이브예금 || iM스마트예금 || iM함께예금 || 굿스타트예금 || 내맘 쏙 정기예금 || 더(The) 레벨업 정기예금 || 더(The) 특판 정기예금 || 미즈월복리정기예금 || 스마일드림 정기예금 (개인/선이자 지급식) || 스마트모아Dream정기예금 || 신한My플러스 정기예금 || 쏠편한 정기예금 || 제주Dream 정기예금 (개인/만기 지급식) || 카카오뱅크 정기예금 || 코드K 정기예금 || 토스뱅크 먼저 이자 받는 정기예금 || 하나의정기예금 || 헤이(Hey)정기예금</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2170,8 +2160,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>BEST고정금리모기지론 || BNK357금리안심모기지론 || BNK모바일주택담보대출 || IBK주택담보대출 || JB전세자금대출 || KB스타 아파트담보대출 혼합금리(주택자금) || KJB셀렉트 주택담보대출 || NH주택담보대출 || ONE주택담보대출 || SH으뜸모기지론 || 개인신용대출(신규대출취급중단)(일반신용대출) || 금리safe모기지론 || 산은 주택대출
-(생활자금) || 신한주택대출 || 신한주택대출(아파트) || 아파트담보대출(구입) || 아파트담보대출(일반) || 우리부동산론 || 우리아파트론 || 주택담보대출 || 집집마다 도움대출II || 채움고정금리모기지론 || 하나원큐아파트론2</t>
+          <t>BEST고정금리모기지론 || BNK357금리안심모기지론 || BNK모바일주택담보대출 || IBK주택담보대출 || JB전세자금대출 || KB스타 아파트담보대출 혼합금리(주택자금) || KJB셀렉트 주택담보대출 || NH주택담보대출 || ONE주택담보대출 || SH으뜸모기지론 || 개인신용대출(신규대출취급중단) || 금리safe모기지론 || 산은 주택대출 (생활자금) || 신한주택대출 || 신한주택대출(아파트) || 아파트담보대출(구입) || 아파트담보대출(일반) || 우리부동산론 || 우리아파트론 || 주택담보대출 || 집집마다 도움대출II || 채움고정금리모기지론 || 하나원큐아파트론2</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2825,8 +2814,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>J정기예금
-(만기지급식)</t>
+          <t>J정기예금 (만기지급식)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2836,8 +2824,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>150,000원을 예치하려는 고객이 제주은행 'J정기예금
-(만기지급식)'의 최소 가입금액 요건을 충족하는가?</t>
+          <t>150,000원을 예치하려는 고객이 제주은행 'J정기예금 (만기지급식)'의 최소 가입금액 요건을 충족하는가?</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2847,8 +2834,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>J정기예금
-(만기지급식) || 30만원 이상</t>
+          <t>J정기예금 (만기지급식) || 30만원 이상</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -3244,8 +3230,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>IBK중기근로자우대적금
-(자유적립식)</t>
+          <t>IBK중기근로자우대적금 (자유적립식)</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -3255,8 +3240,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>중소기업은행 'IBK중기근로자우대적금
-(자유적립식)'의 예금채권을 타인에게 양도하거나 질권을 설정할 수 있는가?</t>
+          <t>중소기업은행 'IBK중기근로자우대적금 (자유적립식)'의 예금채권을 타인에게 양도하거나 질권을 설정할 수 있는가?</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -3506,10 +3490,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>스마일드림 
-정기예금
-(개인/선이자
-지급식)</t>
+          <t>스마일드림 정기예금 (개인/선이자 지급식)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -3519,10 +3500,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>제주은행 '스마일드림 
-정기예금
-(개인/선이자
-지급식)'의 최고 우대금리는 연 0.6%p 이상인가?</t>
+          <t>제주은행 '스마일드림 정기예금 (개인/선이자 지급식)'의 최고 우대금리는 연 0.6%p 이상인가?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -3532,10 +3510,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>스마일드림 
-정기예금
-(개인/선이자
-지급식) || 최고0.3%</t>
+          <t>스마일드림 정기예금 (개인/선이자 지급식) || 최고0.3%</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -3775,10 +3750,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>제주Dream
-정기예금
-(개인/만기
-지급식)</t>
+          <t>제주Dream 정기예금 (개인/만기 지급식)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3788,10 +3760,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>제주은행 '제주Dream
-정기예금
-(개인/만기
-지급식)'의 최고 우대금리는 연 0.2%p 이상인가?</t>
+          <t>제주은행 '제주Dream 정기예금 (개인/만기 지급식)'의 최고 우대금리는 연 0.2%p 이상인가?</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3801,10 +3770,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>제주Dream
-정기예금
-(개인/만기
-지급식) || 최고 연 0.1%p</t>
+          <t>제주Dream 정기예금 (개인/만기 지급식) || 최고 연 0.1%p</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -5032,8 +4998,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>IBK중기근로자우대적금
-(자유적립식)</t>
+          <t>IBK중기근로자우대적금 (자유적립식)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -5043,8 +5008,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>중소기업은행 'IBK중기근로자우대적금
-(자유적립식)'의 최고 우대금리는 연 4.4%p 이상인가?</t>
+          <t>중소기업은행 'IBK중기근로자우대적금 (자유적립식)'의 최고 우대금리는 연 4.4%p 이상인가?</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -5054,8 +5018,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>IBK중기근로자우대적금
-(자유적립식) || 최고 연 2.20%p</t>
+          <t>IBK중기근로자우대적금 (자유적립식) || 최고 연 2.20%p</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -5139,10 +5102,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>제주Dream
-정기예금
-(개인/만기
-지급식)</t>
+          <t>제주Dream 정기예금 (개인/만기 지급식)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -5152,10 +5112,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>제주은행 '제주Dream
-정기예금
-(개인/만기
-지급식)'의 최고 우대금리는 연 0.05%p 이상인가?</t>
+          <t>제주은행 '제주Dream 정기예금 (개인/만기 지급식)'의 최고 우대금리는 연 0.05%p 이상인가?</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -5165,10 +5122,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>제주Dream
-정기예금
-(개인/만기
-지급식) || 최고 연 0.1%p</t>
+          <t>제주Dream 정기예금 (개인/만기 지급식) || 최고 연 0.1%p</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
@@ -5252,10 +5206,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>스마일드림 
-정기예금
-(개인/선이자
-지급식)</t>
+          <t>스마일드림 정기예금 (개인/선이자 지급식)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -5265,10 +5216,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>제주은행 '스마일드림 
-정기예금
-(개인/선이자
-지급식)'의 최고 우대금리는 연 0.15%p 이상인가?</t>
+          <t>제주은행 '스마일드림 정기예금 (개인/선이자 지급식)'의 최고 우대금리는 연 0.15%p 이상인가?</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -5278,10 +5226,7 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>스마일드림 
-정기예금
-(개인/선이자
-지급식) || 최고0.3%</t>
+          <t>스마일드림 정기예금 (개인/선이자 지급식) || 최고0.3%</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
@@ -5365,8 +5310,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>J정기예금
-(만기지급식)</t>
+          <t>J정기예금 (만기지급식)</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -5376,8 +5320,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>제주은행 'J정기예금
-(만기지급식)'의 최고 우대금리는 연 1.0%p 이상인가?</t>
+          <t>제주은행 'J정기예금 (만기지급식)'의 최고 우대금리는 연 1.0%p 이상인가?</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -5387,8 +5330,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>J정기예금
-(만기지급식) || 최고 0.5%p</t>
+          <t>J정기예금 (만기지급식) || 최고 0.5%p</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
@@ -5576,8 +5518,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>IBK중기근로자우대적금
-(자유적립식)</t>
+          <t>IBK중기근로자우대적금 (자유적립식)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -5587,8 +5528,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>중소기업은행 'IBK중기근로자우대적금
-(자유적립식)'의 최고 우대금리는 연 1.1%p 이상인가?</t>
+          <t>중소기업은행 'IBK중기근로자우대적금 (자유적립식)'의 최고 우대금리는 연 1.1%p 이상인가?</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -5598,8 +5538,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>IBK중기근로자우대적금
-(자유적립식) || 최고 연 2.20%p</t>
+          <t>IBK중기근로자우대적금 (자유적립식) || 최고 연 2.20%p</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -5839,8 +5778,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>J정기예금
-(만기지급식)</t>
+          <t>J정기예금 (만기지급식)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -5850,8 +5788,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>제주은행 'J정기예금
-(만기지급식)'의 최고 우대금리는 연 0.25%p 이상인가?</t>
+          <t>제주은행 'J정기예금 (만기지급식)'의 최고 우대금리는 연 0.25%p 이상인가?</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -5861,8 +5798,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>J정기예금
-(만기지급식) || 최고 0.5%p</t>
+          <t>J정기예금 (만기지급식) || 최고 0.5%p</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">

</xml_diff>